<commit_message>
Record selected roof distribution in Rev11 drawing package
</commit_message>
<xml_diff>
--- a/deliverables/rev11/Administration_HVAC_Drawing_Registers_Rev11.xlsx
+++ b/deliverables/rev11/Administration_HVAC_Drawing_Registers_Rev11.xlsx
@@ -929,7 +929,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Roof common mains with 15 independent room drops. OPTION SELECTION PENDING. Actual roof routes and penetrations require structural / architectural coordination.</t>
+          <t>Roof common mains with 15 independent room drops. USER SELECTED ROOF DISTRIBUTION / ROOM DROPS. Actual roof routes and penetrations require structural / architectural coordination.</t>
         </is>
       </c>
     </row>
@@ -41246,7 +41246,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Duct envelope checked; option / structural / OEM selections pending</t>
+          <t>Duct envelope checked; Roof strategy selected; structural / OEM selections pending</t>
         </is>
       </c>
     </row>

</xml_diff>